<commit_message>
mejoras visuales y se agrega campo wat
</commit_message>
<xml_diff>
--- a/templates/11.11.25.xlsx
+++ b/templates/11.11.25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\indicaciones_medicas\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E3C8D6-36F5-45FB-9C4A-DC2810ED5603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9519CBEB-4181-42BB-A1BD-0E8F3AA7DF71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8F26B026-E952-45BF-A1DB-55563CFCC2D9}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8F26B026-E952-45BF-A1DB-55563CFCC2D9}"/>
   </bookViews>
   <sheets>
     <sheet name="Indicaciones médicas" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="90">
   <si>
     <t xml:space="preserve">Fecha </t>
   </si>
@@ -307,6 +307,12 @@
   </si>
   <si>
     <t>VOL HOLLIDAY 60%</t>
+  </si>
+  <si>
+    <t>WAT</t>
+  </si>
+  <si>
+    <t>{{WAT}}</t>
   </si>
 </sst>
 </file>
@@ -317,7 +323,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -421,6 +427,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -436,7 +455,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -665,6 +684,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -672,7 +706,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyBorder="1"/>
@@ -843,10 +877,6 @@
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
@@ -863,16 +893,10 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -882,171 +906,220 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyBorder="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="0" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1129,6 +1202,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Indicaciones médicas"/>
@@ -1507,13 +1581,13 @@
     <row r="2" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="10"/>
       <c r="B2" s="11"/>
-      <c r="C2" s="127" t="s">
+      <c r="C2" s="93" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="128"/>
-      <c r="E2" s="128"/>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
       <c r="I2" s="11"/>
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
@@ -1526,12 +1600,12 @@
     <row r="3" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="10"/>
       <c r="B3" s="11"/>
-      <c r="C3" s="127" t="s">
+      <c r="C3" s="93" t="s">
         <v>46</v>
       </c>
-      <c r="D3" s="128"/>
-      <c r="E3" s="128"/>
-      <c r="F3" s="128"/>
+      <c r="D3" s="94"/>
+      <c r="E3" s="94"/>
+      <c r="F3" s="94"/>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
       <c r="J3" s="11"/>
@@ -1601,11 +1675,11 @@
       <c r="I6" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="J6" s="130" t="s">
+      <c r="J6" s="97" t="s">
         <v>48</v>
       </c>
-      <c r="K6" s="131"/>
-      <c r="L6" s="132"/>
+      <c r="K6" s="98"/>
+      <c r="L6" s="99"/>
       <c r="M6" s="47" t="s">
         <v>8</v>
       </c>
@@ -1623,37 +1697,37 @@
       <c r="A7" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="129" t="s">
+      <c r="B7" s="95" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="104"/>
-      <c r="D7" s="104"/>
-      <c r="E7" s="104"/>
-      <c r="F7" s="104"/>
-      <c r="G7" s="104"/>
-      <c r="H7" s="104"/>
+      <c r="C7" s="89"/>
+      <c r="D7" s="89"/>
+      <c r="E7" s="89"/>
+      <c r="F7" s="89"/>
+      <c r="G7" s="89"/>
+      <c r="H7" s="89"/>
       <c r="I7" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="J7" s="135" t="s">
+      <c r="J7" s="92" t="s">
         <v>51</v>
       </c>
-      <c r="K7" s="103"/>
-      <c r="L7" s="103"/>
-      <c r="M7" s="103"/>
+      <c r="K7" s="88"/>
+      <c r="L7" s="88"/>
+      <c r="M7" s="88"/>
       <c r="N7" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="O7" s="84" t="s">
+      <c r="O7" s="96" t="s">
         <v>52</v>
       </c>
-      <c r="P7" s="103"/>
+      <c r="P7" s="88"/>
     </row>
     <row r="8" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="102" t="s">
+      <c r="A8" s="85" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="103"/>
+      <c r="B8" s="88"/>
       <c r="C8" s="53" t="s">
         <v>15</v>
       </c>
@@ -1666,88 +1740,88 @@
       <c r="F8" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="133" t="s">
+      <c r="G8" s="81" t="s">
         <v>19</v>
       </c>
-      <c r="H8" s="104"/>
-      <c r="I8" s="102" t="s">
+      <c r="H8" s="89"/>
+      <c r="I8" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="J8" s="103"/>
+      <c r="J8" s="88"/>
       <c r="K8" s="56" t="s">
         <v>57</v>
       </c>
       <c r="L8" s="47" t="s">
         <v>75</v>
       </c>
-      <c r="M8" s="134" t="s">
+      <c r="M8" s="90" t="s">
         <v>76</v>
       </c>
-      <c r="N8" s="106"/>
-      <c r="O8" s="106"/>
-      <c r="P8" s="106"/>
+      <c r="N8" s="91"/>
+      <c r="O8" s="91"/>
+      <c r="P8" s="91"/>
     </row>
     <row r="9" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="102" t="s">
+      <c r="A9" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="103"/>
-      <c r="C9" s="91" t="s">
+      <c r="B9" s="88"/>
+      <c r="C9" s="103" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="104"/>
-      <c r="E9" s="104"/>
-      <c r="F9" s="104"/>
-      <c r="G9" s="104"/>
-      <c r="H9" s="104"/>
-      <c r="I9" s="104"/>
-      <c r="J9" s="104"/>
-      <c r="K9" s="104"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="89"/>
+      <c r="F9" s="89"/>
+      <c r="G9" s="89"/>
+      <c r="H9" s="89"/>
+      <c r="I9" s="89"/>
+      <c r="J9" s="89"/>
+      <c r="K9" s="89"/>
       <c r="L9" s="57"/>
-      <c r="M9" s="110"/>
-      <c r="N9" s="103"/>
-      <c r="O9" s="103"/>
-      <c r="P9" s="103"/>
+      <c r="M9" s="104"/>
+      <c r="N9" s="88"/>
+      <c r="O9" s="88"/>
+      <c r="P9" s="88"/>
     </row>
     <row r="10" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="102" t="s">
+      <c r="A10" s="85" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="103"/>
-      <c r="C10" s="91" t="s">
+      <c r="B10" s="88"/>
+      <c r="C10" s="103" t="s">
         <v>24</v>
       </c>
-      <c r="D10" s="104"/>
-      <c r="E10" s="104"/>
-      <c r="F10" s="104"/>
-      <c r="G10" s="104"/>
-      <c r="H10" s="104"/>
-      <c r="I10" s="104"/>
-      <c r="J10" s="104"/>
-      <c r="K10" s="104"/>
-      <c r="L10" s="104"/>
-      <c r="M10" s="104"/>
-      <c r="N10" s="104"/>
-      <c r="O10" s="104"/>
-      <c r="P10" s="104"/>
+      <c r="D10" s="89"/>
+      <c r="E10" s="89"/>
+      <c r="F10" s="89"/>
+      <c r="G10" s="89"/>
+      <c r="H10" s="89"/>
+      <c r="I10" s="89"/>
+      <c r="J10" s="89"/>
+      <c r="K10" s="89"/>
+      <c r="L10" s="89"/>
+      <c r="M10" s="89"/>
+      <c r="N10" s="89"/>
+      <c r="O10" s="89"/>
+      <c r="P10" s="89"/>
     </row>
     <row r="11" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="105" t="s">
+      <c r="A11" s="116" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="106"/>
+      <c r="B11" s="91"/>
       <c r="C11" s="46" t="s">
         <v>53</v>
       </c>
-      <c r="D11" s="105" t="s">
+      <c r="D11" s="116" t="s">
         <v>77</v>
       </c>
-      <c r="E11" s="106"/>
+      <c r="E11" s="91"/>
       <c r="F11" s="54" t="s">
         <v>78</v>
       </c>
-      <c r="G11" s="102"/>
-      <c r="H11" s="103"/>
+      <c r="G11" s="85"/>
+      <c r="H11" s="88"/>
       <c r="I11" s="47"/>
       <c r="J11" s="50" t="s">
         <v>26</v>
@@ -1764,16 +1838,16 @@
       <c r="N11" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="O11" s="124" t="s">
+      <c r="O11" s="115" t="s">
         <v>79</v>
       </c>
-      <c r="P11" s="104"/>
+      <c r="P11" s="89"/>
     </row>
     <row r="12" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="105" t="s">
+      <c r="A12" s="116" t="s">
         <v>87</v>
       </c>
-      <c r="B12" s="106"/>
+      <c r="B12" s="91"/>
       <c r="C12" s="60" t="s">
         <v>81</v>
       </c>
@@ -1802,38 +1876,38 @@
       <c r="D13" s="62"/>
       <c r="E13" s="62"/>
       <c r="F13" s="62"/>
-      <c r="G13" s="107"/>
-      <c r="H13" s="108"/>
-      <c r="I13" s="108"/>
-      <c r="J13" s="108"/>
-      <c r="K13" s="108"/>
-      <c r="L13" s="108"/>
-      <c r="M13" s="108"/>
-      <c r="N13" s="108"/>
-      <c r="O13" s="108"/>
-      <c r="P13" s="109"/>
+      <c r="G13" s="100"/>
+      <c r="H13" s="101"/>
+      <c r="I13" s="101"/>
+      <c r="J13" s="101"/>
+      <c r="K13" s="101"/>
+      <c r="L13" s="101"/>
+      <c r="M13" s="101"/>
+      <c r="N13" s="101"/>
+      <c r="O13" s="101"/>
+      <c r="P13" s="102"/>
     </row>
     <row r="14" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="66"/>
       <c r="B14" s="67" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="123" t="s">
+      <c r="C14" s="112" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="92"/>
-      <c r="E14" s="92"/>
-      <c r="F14" s="92"/>
-      <c r="G14" s="92"/>
-      <c r="H14" s="92"/>
-      <c r="I14" s="92"/>
-      <c r="J14" s="92"/>
-      <c r="K14" s="92"/>
-      <c r="L14" s="92"/>
-      <c r="M14" s="92"/>
-      <c r="N14" s="92"/>
-      <c r="O14" s="92"/>
-      <c r="P14" s="93"/>
+      <c r="D14" s="113"/>
+      <c r="E14" s="113"/>
+      <c r="F14" s="113"/>
+      <c r="G14" s="113"/>
+      <c r="H14" s="113"/>
+      <c r="I14" s="113"/>
+      <c r="J14" s="113"/>
+      <c r="K14" s="113"/>
+      <c r="L14" s="113"/>
+      <c r="M14" s="113"/>
+      <c r="N14" s="113"/>
+      <c r="O14" s="113"/>
+      <c r="P14" s="114"/>
     </row>
     <row r="15" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="68"/>
@@ -1843,25 +1917,25 @@
       <c r="C15" s="69" t="s">
         <v>59</v>
       </c>
-      <c r="D15" s="69" t="s">
+      <c r="D15" s="140" t="s">
         <v>60</v>
       </c>
-      <c r="E15" s="69" t="s">
+      <c r="E15" s="140" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="70" t="s">
+      <c r="F15" s="141" t="s">
         <v>61</v>
       </c>
-      <c r="G15" s="69" t="s">
+      <c r="G15" s="140" t="s">
         <v>33</v>
       </c>
-      <c r="H15" s="70" t="s">
+      <c r="H15" s="141" t="s">
         <v>62</v>
       </c>
-      <c r="I15" s="69" t="s">
+      <c r="I15" s="140" t="s">
         <v>34</v>
       </c>
-      <c r="J15" s="69" t="s">
+      <c r="J15" s="140" t="s">
         <v>63</v>
       </c>
       <c r="K15" s="69"/>
@@ -1871,233 +1945,237 @@
       <c r="O15" s="52"/>
       <c r="P15" s="52"/>
     </row>
-    <row r="16" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="53"/>
       <c r="B16" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="125" t="s">
+      <c r="C16" s="147" t="s">
         <v>65</v>
       </c>
-      <c r="D16" s="88"/>
-      <c r="E16" s="88"/>
-      <c r="F16" s="89"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="72"/>
-      <c r="I16" s="73" t="s">
+      <c r="D16" s="145"/>
+      <c r="E16" s="145"/>
+      <c r="F16" s="146"/>
+      <c r="G16" s="70"/>
+      <c r="H16" s="71"/>
+      <c r="I16" s="142" t="s">
         <v>36</v>
       </c>
-      <c r="J16" s="72" t="s">
+      <c r="J16" s="143" t="s">
         <v>64</v>
       </c>
-      <c r="K16" s="73"/>
-      <c r="L16" s="72"/>
-      <c r="M16" s="74"/>
-      <c r="N16" s="72"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="75"/>
-    </row>
-    <row r="17" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="133"/>
-      <c r="B17" s="76" t="s">
+      <c r="K16" s="72"/>
+      <c r="L16" s="71"/>
+      <c r="M16" s="73"/>
+      <c r="N16" s="71"/>
+      <c r="O16" s="74"/>
+      <c r="P16" s="74"/>
+    </row>
+    <row r="17" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="81"/>
+      <c r="B17" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="C17" s="126" t="s">
+      <c r="C17" s="144" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="88"/>
-      <c r="E17" s="88"/>
-      <c r="F17" s="88"/>
-      <c r="G17" s="88"/>
-      <c r="H17" s="88"/>
-      <c r="I17" s="88"/>
-      <c r="J17" s="88"/>
-      <c r="K17" s="88"/>
-      <c r="L17" s="88"/>
-      <c r="M17" s="88"/>
-      <c r="N17" s="88"/>
-      <c r="O17" s="88"/>
-      <c r="P17" s="89"/>
+      <c r="D17" s="145"/>
+      <c r="E17" s="145"/>
+      <c r="F17" s="145"/>
+      <c r="G17" s="145"/>
+      <c r="H17" s="145"/>
+      <c r="I17" s="145"/>
+      <c r="J17" s="145"/>
+      <c r="K17" s="145"/>
+      <c r="L17" s="145"/>
+      <c r="M17" s="145"/>
+      <c r="N17" s="145"/>
+      <c r="O17" s="145"/>
+      <c r="P17" s="146"/>
     </row>
     <row r="18" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="138"/>
-      <c r="B18" s="84" t="s">
+      <c r="A18" s="82"/>
+      <c r="B18" s="96" t="s">
         <v>38</v>
       </c>
-      <c r="C18" s="85"/>
-      <c r="D18" s="85"/>
-      <c r="E18" s="85"/>
-      <c r="F18" s="85"/>
-      <c r="G18" s="85"/>
-      <c r="H18" s="85"/>
-      <c r="I18" s="85"/>
-      <c r="J18" s="85"/>
-      <c r="K18" s="85"/>
-      <c r="L18" s="85"/>
-      <c r="M18" s="85"/>
-      <c r="N18" s="85"/>
-      <c r="O18" s="85"/>
-      <c r="P18" s="86"/>
+      <c r="C18" s="86"/>
+      <c r="D18" s="86"/>
+      <c r="E18" s="86"/>
+      <c r="F18" s="86"/>
+      <c r="G18" s="86"/>
+      <c r="H18" s="86"/>
+      <c r="I18" s="86"/>
+      <c r="J18" s="86"/>
+      <c r="K18" s="86"/>
+      <c r="L18" s="86"/>
+      <c r="M18" s="86"/>
+      <c r="N18" s="86"/>
+      <c r="O18" s="86"/>
+      <c r="P18" s="87"/>
     </row>
     <row r="19" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="87" t="s">
+      <c r="B19" s="117" t="s">
         <v>80</v>
       </c>
-      <c r="C19" s="88"/>
-      <c r="D19" s="88"/>
-      <c r="E19" s="88"/>
-      <c r="F19" s="89"/>
-      <c r="G19" s="90"/>
-      <c r="H19" s="88"/>
-      <c r="I19" s="88"/>
-      <c r="J19" s="88"/>
-      <c r="K19" s="88"/>
-      <c r="L19" s="88"/>
-      <c r="M19" s="88"/>
-      <c r="N19" s="88"/>
-      <c r="O19" s="88"/>
-      <c r="P19" s="89"/>
+      <c r="C19" s="106"/>
+      <c r="D19" s="106"/>
+      <c r="E19" s="106"/>
+      <c r="F19" s="107"/>
+      <c r="G19" s="118"/>
+      <c r="H19" s="106"/>
+      <c r="I19" s="106"/>
+      <c r="J19" s="106"/>
+      <c r="K19" s="106"/>
+      <c r="L19" s="106"/>
+      <c r="M19" s="106"/>
+      <c r="N19" s="106"/>
+      <c r="O19" s="106"/>
+      <c r="P19" s="107"/>
     </row>
     <row r="20" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="14"/>
-      <c r="B20" s="91"/>
-      <c r="C20" s="92"/>
-      <c r="D20" s="92"/>
-      <c r="E20" s="92"/>
-      <c r="F20" s="92"/>
-      <c r="G20" s="92"/>
-      <c r="H20" s="92"/>
-      <c r="I20" s="92"/>
-      <c r="J20" s="92"/>
-      <c r="K20" s="92"/>
-      <c r="L20" s="92"/>
-      <c r="M20" s="92"/>
-      <c r="N20" s="92"/>
-      <c r="O20" s="92"/>
-      <c r="P20" s="93"/>
-    </row>
-    <row r="21" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="103"/>
+      <c r="C20" s="113"/>
+      <c r="D20" s="113"/>
+      <c r="E20" s="113"/>
+      <c r="F20" s="113"/>
+      <c r="G20" s="113"/>
+      <c r="H20" s="113"/>
+      <c r="I20" s="113"/>
+      <c r="J20" s="113"/>
+      <c r="K20" s="113"/>
+      <c r="L20" s="113"/>
+      <c r="M20" s="113"/>
+      <c r="N20" s="113"/>
+      <c r="O20" s="113"/>
+      <c r="P20" s="114"/>
+    </row>
+    <row r="21" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="111" t="s">
+      <c r="B21" s="128" t="s">
         <v>67</v>
       </c>
-      <c r="C21" s="108"/>
-      <c r="D21" s="108"/>
-      <c r="E21" s="108"/>
-      <c r="F21" s="108"/>
-      <c r="G21" s="108"/>
-      <c r="H21" s="108"/>
-      <c r="I21" s="108"/>
-      <c r="J21" s="108"/>
-      <c r="K21" s="108"/>
-      <c r="L21" s="108"/>
-      <c r="M21" s="108"/>
-      <c r="N21" s="108"/>
-      <c r="O21" s="108"/>
-      <c r="P21" s="109"/>
-    </row>
-    <row r="22" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C21" s="132"/>
+      <c r="D21" s="132"/>
+      <c r="E21" s="132"/>
+      <c r="F21" s="132"/>
+      <c r="G21" s="132"/>
+      <c r="H21" s="132"/>
+      <c r="I21" s="132"/>
+      <c r="J21" s="132"/>
+      <c r="K21" s="132"/>
+      <c r="L21" s="132"/>
+      <c r="M21" s="132"/>
+      <c r="N21" s="132"/>
+      <c r="O21" s="132"/>
+      <c r="P21" s="133"/>
+    </row>
+    <row r="22" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="B22" s="112" t="s">
+      <c r="B22" s="127" t="s">
         <v>68</v>
       </c>
-      <c r="C22" s="113"/>
-      <c r="D22" s="113"/>
-      <c r="E22" s="113"/>
-      <c r="F22" s="114"/>
-      <c r="G22" s="115"/>
-      <c r="H22" s="88"/>
-      <c r="I22" s="88"/>
-      <c r="J22" s="88"/>
-      <c r="K22" s="88"/>
-      <c r="L22" s="88"/>
-      <c r="M22" s="88"/>
-      <c r="N22" s="88"/>
-      <c r="O22" s="88"/>
-      <c r="P22" s="89"/>
-    </row>
-    <row r="23" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C22" s="130"/>
+      <c r="D22" s="130"/>
+      <c r="E22" s="130"/>
+      <c r="F22" s="131"/>
+      <c r="G22" s="105"/>
+      <c r="H22" s="106"/>
+      <c r="I22" s="106"/>
+      <c r="J22" s="106"/>
+      <c r="K22" s="106"/>
+      <c r="L22" s="106"/>
+      <c r="M22" s="106"/>
+      <c r="N22" s="106"/>
+      <c r="O22" s="106"/>
+      <c r="P22" s="107"/>
+    </row>
+    <row r="23" spans="1:16" ht="27.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B23" s="116" t="s">
+      <c r="B23" s="129" t="s">
         <v>69</v>
       </c>
-      <c r="C23" s="117"/>
-      <c r="D23" s="117"/>
-      <c r="E23" s="117"/>
-      <c r="F23" s="118"/>
-      <c r="G23" s="94" t="s">
+      <c r="C23" s="134"/>
+      <c r="D23" s="134"/>
+      <c r="E23" s="134"/>
+      <c r="F23" s="135"/>
+      <c r="G23" s="119" t="s">
         <v>85</v>
       </c>
-      <c r="H23" s="95"/>
-      <c r="I23" s="77" t="s">
+      <c r="H23" s="120"/>
+      <c r="I23" s="136" t="s">
         <v>70</v>
       </c>
-      <c r="J23" s="78"/>
-      <c r="K23" s="94" t="s">
+      <c r="J23" s="76"/>
+      <c r="K23" s="119" t="s">
         <v>86</v>
       </c>
-      <c r="L23" s="95"/>
-      <c r="M23" s="94" t="s">
+      <c r="L23" s="120"/>
+      <c r="M23" s="137" t="s">
         <v>71</v>
       </c>
-      <c r="N23" s="95"/>
-      <c r="O23" s="79"/>
-      <c r="P23" s="80"/>
+      <c r="N23" s="138"/>
+      <c r="O23" s="77" t="s">
+        <v>88</v>
+      </c>
+      <c r="P23" s="139" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20"/>
-      <c r="B24" s="119"/>
-      <c r="C24" s="120"/>
-      <c r="D24" s="120"/>
-      <c r="E24" s="120"/>
-      <c r="F24" s="120"/>
-      <c r="G24" s="121"/>
-      <c r="H24" s="121"/>
-      <c r="I24" s="120"/>
-      <c r="J24" s="121"/>
-      <c r="K24" s="120"/>
-      <c r="L24" s="120"/>
-      <c r="M24" s="120"/>
-      <c r="N24" s="120"/>
-      <c r="O24" s="120"/>
-      <c r="P24" s="122"/>
+      <c r="B24" s="108"/>
+      <c r="C24" s="109"/>
+      <c r="D24" s="109"/>
+      <c r="E24" s="109"/>
+      <c r="F24" s="109"/>
+      <c r="G24" s="110"/>
+      <c r="H24" s="110"/>
+      <c r="I24" s="109"/>
+      <c r="J24" s="110"/>
+      <c r="K24" s="109"/>
+      <c r="L24" s="109"/>
+      <c r="M24" s="109"/>
+      <c r="N24" s="109"/>
+      <c r="O24" s="109"/>
+      <c r="P24" s="111"/>
     </row>
     <row r="25" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="35"/>
-      <c r="B25" s="99"/>
-      <c r="C25" s="100"/>
-      <c r="D25" s="100"/>
-      <c r="E25" s="100"/>
-      <c r="F25" s="100"/>
-      <c r="G25" s="100"/>
-      <c r="H25" s="100"/>
-      <c r="I25" s="100"/>
-      <c r="J25" s="100"/>
-      <c r="K25" s="100"/>
-      <c r="L25" s="100"/>
-      <c r="M25" s="100"/>
-      <c r="N25" s="100"/>
-      <c r="O25" s="100"/>
-      <c r="P25" s="101"/>
+      <c r="B25" s="124"/>
+      <c r="C25" s="125"/>
+      <c r="D25" s="125"/>
+      <c r="E25" s="125"/>
+      <c r="F25" s="125"/>
+      <c r="G25" s="125"/>
+      <c r="H25" s="125"/>
+      <c r="I25" s="125"/>
+      <c r="J25" s="125"/>
+      <c r="K25" s="125"/>
+      <c r="L25" s="125"/>
+      <c r="M25" s="125"/>
+      <c r="N25" s="125"/>
+      <c r="O25" s="125"/>
+      <c r="P25" s="126"/>
     </row>
     <row r="26" spans="1:16" ht="27.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="21"/>
-      <c r="B26" s="96" t="s">
+      <c r="B26" s="121" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="97"/>
-      <c r="D26" s="97"/>
-      <c r="E26" s="97"/>
-      <c r="F26" s="98"/>
+      <c r="C26" s="122"/>
+      <c r="D26" s="122"/>
+      <c r="E26" s="122"/>
+      <c r="F26" s="123"/>
       <c r="G26" s="42"/>
       <c r="H26" s="40"/>
       <c r="I26" s="40"/>
@@ -2113,11 +2191,11 @@
       <c r="A27" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B27" s="81" t="s">
+      <c r="B27" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C27" s="82"/>
-      <c r="D27" s="83"/>
+      <c r="C27" s="79"/>
+      <c r="D27" s="80"/>
       <c r="E27" s="38"/>
       <c r="F27" s="22"/>
       <c r="G27" s="23"/>
@@ -2161,11 +2239,11 @@
       <c r="A29" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="81" t="s">
+      <c r="B29" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C29" s="82"/>
-      <c r="D29" s="83"/>
+      <c r="C29" s="79"/>
+      <c r="D29" s="80"/>
       <c r="E29" s="27"/>
       <c r="F29" s="28"/>
       <c r="G29" s="29"/>
@@ -2209,11 +2287,11 @@
       <c r="A31" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B31" s="81" t="s">
+      <c r="B31" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="82"/>
-      <c r="D31" s="83"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="80"/>
       <c r="E31" s="27"/>
       <c r="F31" s="28"/>
       <c r="G31" s="29"/>
@@ -2257,11 +2335,11 @@
       <c r="A33" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B33" s="81" t="s">
+      <c r="B33" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C33" s="82"/>
-      <c r="D33" s="83"/>
+      <c r="C33" s="79"/>
+      <c r="D33" s="80"/>
       <c r="E33" s="27"/>
       <c r="F33" s="28"/>
       <c r="G33" s="29"/>
@@ -2305,11 +2383,11 @@
       <c r="A35" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B35" s="81" t="s">
+      <c r="B35" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C35" s="82"/>
-      <c r="D35" s="83"/>
+      <c r="C35" s="79"/>
+      <c r="D35" s="80"/>
       <c r="E35" s="27"/>
       <c r="F35" s="28"/>
       <c r="G35" s="29"/>
@@ -2353,11 +2431,11 @@
       <c r="A37" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B37" s="81" t="s">
+      <c r="B37" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="82"/>
-      <c r="D37" s="83"/>
+      <c r="C37" s="79"/>
+      <c r="D37" s="80"/>
       <c r="E37" s="27"/>
       <c r="F37" s="28"/>
       <c r="G37" s="29"/>
@@ -2401,11 +2479,11 @@
       <c r="A39" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B39" s="81" t="s">
+      <c r="B39" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C39" s="82"/>
-      <c r="D39" s="83"/>
+      <c r="C39" s="79"/>
+      <c r="D39" s="80"/>
       <c r="E39" s="27"/>
       <c r="F39" s="28"/>
       <c r="G39" s="29"/>
@@ -2449,11 +2527,11 @@
       <c r="A41" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B41" s="81" t="s">
+      <c r="B41" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C41" s="82"/>
-      <c r="D41" s="83"/>
+      <c r="C41" s="79"/>
+      <c r="D41" s="80"/>
       <c r="E41" s="27"/>
       <c r="F41" s="28"/>
       <c r="G41" s="29"/>
@@ -2497,11 +2575,11 @@
       <c r="A43" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B43" s="81" t="s">
+      <c r="B43" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C43" s="82"/>
-      <c r="D43" s="83"/>
+      <c r="C43" s="79"/>
+      <c r="D43" s="80"/>
       <c r="E43" s="27"/>
       <c r="F43" s="28"/>
       <c r="G43" s="29"/>
@@ -2545,11 +2623,11 @@
       <c r="A45" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B45" s="81" t="s">
+      <c r="B45" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C45" s="82"/>
-      <c r="D45" s="83"/>
+      <c r="C45" s="79"/>
+      <c r="D45" s="80"/>
       <c r="E45" s="27"/>
       <c r="F45" s="28"/>
       <c r="G45" s="29"/>
@@ -2593,11 +2671,11 @@
       <c r="A47" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="81" t="s">
+      <c r="B47" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C47" s="82"/>
-      <c r="D47" s="83"/>
+      <c r="C47" s="79"/>
+      <c r="D47" s="80"/>
       <c r="E47" s="27"/>
       <c r="F47" s="28"/>
       <c r="G47" s="29"/>
@@ -2641,11 +2719,11 @@
       <c r="A49" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B49" s="81" t="s">
+      <c r="B49" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C49" s="82"/>
-      <c r="D49" s="83"/>
+      <c r="C49" s="79"/>
+      <c r="D49" s="80"/>
       <c r="E49" s="27"/>
       <c r="F49" s="28"/>
       <c r="G49" s="29"/>
@@ -2689,11 +2767,11 @@
       <c r="A51" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B51" s="81" t="s">
+      <c r="B51" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C51" s="82"/>
-      <c r="D51" s="83"/>
+      <c r="C51" s="79"/>
+      <c r="D51" s="80"/>
       <c r="E51" s="27"/>
       <c r="F51" s="28"/>
       <c r="G51" s="29"/>
@@ -2737,11 +2815,11 @@
       <c r="A53" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B53" s="81" t="s">
+      <c r="B53" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C53" s="82"/>
-      <c r="D53" s="83"/>
+      <c r="C53" s="79"/>
+      <c r="D53" s="80"/>
       <c r="E53" s="27"/>
       <c r="F53" s="28"/>
       <c r="G53" s="29"/>
@@ -2785,11 +2863,11 @@
       <c r="A55" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B55" s="81" t="s">
+      <c r="B55" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C55" s="82"/>
-      <c r="D55" s="83"/>
+      <c r="C55" s="79"/>
+      <c r="D55" s="80"/>
       <c r="E55" s="27"/>
       <c r="F55" s="28"/>
       <c r="G55" s="29"/>
@@ -2833,21 +2911,21 @@
       <c r="A57" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B57" s="102"/>
-      <c r="C57" s="85"/>
-      <c r="D57" s="86"/>
+      <c r="B57" s="85"/>
+      <c r="C57" s="86"/>
+      <c r="D57" s="87"/>
       <c r="E57" s="32"/>
       <c r="F57" s="33"/>
-      <c r="G57" s="136" t="s">
+      <c r="G57" s="83" t="s">
         <v>44</v>
       </c>
-      <c r="H57" s="137"/>
-      <c r="I57" s="137"/>
-      <c r="J57" s="137"/>
-      <c r="K57" s="137"/>
-      <c r="L57" s="137"/>
-      <c r="M57" s="137"/>
-      <c r="N57" s="137"/>
+      <c r="H57" s="84"/>
+      <c r="I57" s="84"/>
+      <c r="J57" s="84"/>
+      <c r="K57" s="84"/>
+      <c r="L57" s="84"/>
+      <c r="M57" s="84"/>
+      <c r="N57" s="84"/>
       <c r="O57" s="36"/>
       <c r="P57" s="37"/>
     </row>
@@ -2855,11 +2933,11 @@
       <c r="A58" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B58" s="81" t="s">
+      <c r="B58" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C58" s="82"/>
-      <c r="D58" s="83"/>
+      <c r="C58" s="79"/>
+      <c r="D58" s="80"/>
       <c r="E58" s="27"/>
       <c r="F58" s="28"/>
       <c r="G58" s="29"/>
@@ -2903,11 +2981,11 @@
       <c r="A60" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B60" s="81" t="s">
+      <c r="B60" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C60" s="82"/>
-      <c r="D60" s="83"/>
+      <c r="C60" s="79"/>
+      <c r="D60" s="80"/>
       <c r="E60" s="27"/>
       <c r="F60" s="28"/>
       <c r="G60" s="29"/>
@@ -2951,11 +3029,11 @@
       <c r="A62" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B62" s="81" t="s">
+      <c r="B62" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C62" s="82"/>
-      <c r="D62" s="83"/>
+      <c r="C62" s="79"/>
+      <c r="D62" s="80"/>
       <c r="E62" s="27"/>
       <c r="F62" s="28"/>
       <c r="G62" s="29"/>
@@ -2999,11 +3077,11 @@
       <c r="A64" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B64" s="81" t="s">
+      <c r="B64" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C64" s="82"/>
-      <c r="D64" s="83"/>
+      <c r="C64" s="79"/>
+      <c r="D64" s="80"/>
       <c r="E64" s="27"/>
       <c r="F64" s="28"/>
       <c r="G64" s="29"/>
@@ -3047,11 +3125,11 @@
       <c r="A66" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B66" s="81" t="s">
+      <c r="B66" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C66" s="82"/>
-      <c r="D66" s="83"/>
+      <c r="C66" s="79"/>
+      <c r="D66" s="80"/>
       <c r="E66" s="27"/>
       <c r="F66" s="28"/>
       <c r="G66" s="29"/>
@@ -3095,11 +3173,11 @@
       <c r="A68" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B68" s="81" t="s">
+      <c r="B68" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C68" s="82"/>
-      <c r="D68" s="83"/>
+      <c r="C68" s="79"/>
+      <c r="D68" s="80"/>
       <c r="E68" s="27"/>
       <c r="F68" s="28"/>
       <c r="G68" s="29"/>
@@ -3143,11 +3221,11 @@
       <c r="A70" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B70" s="81" t="s">
+      <c r="B70" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C70" s="82"/>
-      <c r="D70" s="83"/>
+      <c r="C70" s="79"/>
+      <c r="D70" s="80"/>
       <c r="E70" s="27"/>
       <c r="F70" s="28"/>
       <c r="G70" s="29"/>
@@ -3191,11 +3269,11 @@
       <c r="A72" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B72" s="81" t="s">
+      <c r="B72" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C72" s="82"/>
-      <c r="D72" s="83"/>
+      <c r="C72" s="79"/>
+      <c r="D72" s="80"/>
       <c r="E72" s="27"/>
       <c r="F72" s="28"/>
       <c r="G72" s="29"/>
@@ -3239,11 +3317,11 @@
       <c r="A74" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B74" s="81" t="s">
+      <c r="B74" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C74" s="82"/>
-      <c r="D74" s="83"/>
+      <c r="C74" s="79"/>
+      <c r="D74" s="80"/>
       <c r="E74" s="27"/>
       <c r="F74" s="28"/>
       <c r="G74" s="29"/>
@@ -3287,11 +3365,11 @@
       <c r="A76" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B76" s="81" t="s">
+      <c r="B76" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C76" s="82"/>
-      <c r="D76" s="83"/>
+      <c r="C76" s="79"/>
+      <c r="D76" s="80"/>
       <c r="E76" s="27"/>
       <c r="F76" s="28"/>
       <c r="G76" s="29"/>
@@ -3335,11 +3413,11 @@
       <c r="A78" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B78" s="81" t="s">
+      <c r="B78" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C78" s="82"/>
-      <c r="D78" s="83"/>
+      <c r="C78" s="79"/>
+      <c r="D78" s="80"/>
       <c r="E78" s="27"/>
       <c r="F78" s="28"/>
       <c r="G78" s="29"/>
@@ -3383,11 +3461,11 @@
       <c r="A80" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B80" s="81" t="s">
+      <c r="B80" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C80" s="82"/>
-      <c r="D80" s="83"/>
+      <c r="C80" s="79"/>
+      <c r="D80" s="80"/>
       <c r="E80" s="27"/>
       <c r="F80" s="28"/>
       <c r="G80" s="29"/>
@@ -3431,11 +3509,11 @@
       <c r="A82" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B82" s="81" t="s">
+      <c r="B82" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C82" s="82"/>
-      <c r="D82" s="83"/>
+      <c r="C82" s="79"/>
+      <c r="D82" s="80"/>
       <c r="E82" s="27"/>
       <c r="F82" s="28"/>
       <c r="G82" s="29"/>
@@ -3479,11 +3557,11 @@
       <c r="A84" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B84" s="81" t="s">
+      <c r="B84" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C84" s="82"/>
-      <c r="D84" s="83"/>
+      <c r="C84" s="79"/>
+      <c r="D84" s="80"/>
       <c r="E84" s="27"/>
       <c r="F84" s="28"/>
       <c r="G84" s="29"/>
@@ -3527,11 +3605,11 @@
       <c r="A86" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B86" s="81" t="s">
+      <c r="B86" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C86" s="82"/>
-      <c r="D86" s="83"/>
+      <c r="C86" s="79"/>
+      <c r="D86" s="80"/>
       <c r="E86" s="27"/>
       <c r="F86" s="28"/>
       <c r="G86" s="29"/>
@@ -3575,11 +3653,11 @@
       <c r="A88" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B88" s="81" t="s">
+      <c r="B88" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C88" s="82"/>
-      <c r="D88" s="83"/>
+      <c r="C88" s="79"/>
+      <c r="D88" s="80"/>
       <c r="E88" s="27"/>
       <c r="F88" s="28"/>
       <c r="G88" s="29"/>
@@ -3623,11 +3701,11 @@
       <c r="A90" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B90" s="81" t="s">
+      <c r="B90" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C90" s="82"/>
-      <c r="D90" s="83"/>
+      <c r="C90" s="79"/>
+      <c r="D90" s="80"/>
       <c r="E90" s="27"/>
       <c r="F90" s="28"/>
       <c r="G90" s="29"/>
@@ -3671,11 +3749,11 @@
       <c r="A92" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B92" s="81" t="s">
+      <c r="B92" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C92" s="82"/>
-      <c r="D92" s="83"/>
+      <c r="C92" s="79"/>
+      <c r="D92" s="80"/>
       <c r="E92" s="27"/>
       <c r="F92" s="28"/>
       <c r="G92" s="29"/>
@@ -3719,11 +3797,11 @@
       <c r="A94" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B94" s="81" t="s">
+      <c r="B94" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C94" s="82"/>
-      <c r="D94" s="83"/>
+      <c r="C94" s="79"/>
+      <c r="D94" s="80"/>
       <c r="E94" s="27"/>
       <c r="F94" s="28"/>
       <c r="G94" s="29"/>
@@ -3767,11 +3845,11 @@
       <c r="A96" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B96" s="81" t="s">
+      <c r="B96" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C96" s="82"/>
-      <c r="D96" s="83"/>
+      <c r="C96" s="79"/>
+      <c r="D96" s="80"/>
       <c r="E96" s="27"/>
       <c r="F96" s="28"/>
       <c r="G96" s="29"/>
@@ -3815,11 +3893,11 @@
       <c r="A98" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B98" s="81" t="s">
+      <c r="B98" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C98" s="82"/>
-      <c r="D98" s="83"/>
+      <c r="C98" s="79"/>
+      <c r="D98" s="80"/>
       <c r="E98" s="27"/>
       <c r="F98" s="28"/>
       <c r="G98" s="29"/>
@@ -3863,11 +3941,11 @@
       <c r="A100" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="B100" s="81" t="s">
+      <c r="B100" s="78" t="s">
         <v>72</v>
       </c>
-      <c r="C100" s="82"/>
-      <c r="D100" s="83"/>
+      <c r="C100" s="79"/>
+      <c r="D100" s="80"/>
       <c r="E100" s="27"/>
       <c r="F100" s="28"/>
       <c r="G100" s="29"/>
@@ -4089,6 +4167,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B18:P18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="G19:P19"/>
+    <mergeCell ref="B20:P20"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="B26:F26"/>
+    <mergeCell ref="B25:P25"/>
+    <mergeCell ref="M23:N23"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:P10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G13:P13"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="C9:K9"/>
+    <mergeCell ref="M9:P9"/>
+    <mergeCell ref="B21:P21"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="G22:P22"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B24:P24"/>
+    <mergeCell ref="B27:D27"/>
+    <mergeCell ref="C14:P14"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C17:P17"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="C3:F3"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="J6:L6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="M8:P8"/>
+    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="G57:N57"/>
+    <mergeCell ref="B41:D41"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="B62:D62"/>
+    <mergeCell ref="B64:D64"/>
     <mergeCell ref="B98:D98"/>
     <mergeCell ref="B100:D100"/>
     <mergeCell ref="A17:A18"/>
@@ -4105,68 +4245,6 @@
     <mergeCell ref="B86:D86"/>
     <mergeCell ref="B70:D70"/>
     <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B74:D74"/>
-    <mergeCell ref="B76:D76"/>
-    <mergeCell ref="B78:D78"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B62:D62"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="G57:N57"/>
-    <mergeCell ref="B41:D41"/>
-    <mergeCell ref="B43:D43"/>
-    <mergeCell ref="B45:D45"/>
-    <mergeCell ref="B47:D47"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="M8:P8"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="C3:F3"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="J6:L6"/>
-    <mergeCell ref="G13:P13"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="C9:K9"/>
-    <mergeCell ref="M9:P9"/>
-    <mergeCell ref="B21:P21"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="G22:P22"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B24:P24"/>
-    <mergeCell ref="B27:D27"/>
-    <mergeCell ref="C14:P14"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C17:P17"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="C10:P10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B18:P18"/>
-    <mergeCell ref="B19:F19"/>
-    <mergeCell ref="G19:P19"/>
-    <mergeCell ref="B20:P20"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="B26:F26"/>
-    <mergeCell ref="B25:P25"/>
-    <mergeCell ref="M23:N23"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup scale="47" fitToHeight="2" orientation="portrait" r:id="rId1"/>

</xml_diff>